<commit_message>
fix import user resignation
</commit_message>
<xml_diff>
--- a/public/template_excel/nghi_viec.xlsx
+++ b/public/template_excel/nghi_viec.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguyenviet\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\FESP\fe-service-portal\public\template_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46CE90C2-855F-4CDB-A00B-E257154690D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51026347-0AD5-4AE2-8F0D-D2221F9071AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>stt</t>
   </si>
@@ -40,6 +40,21 @@
   </si>
   <si>
     <t>ly_do_nghi</t>
+  </si>
+  <si>
+    <t>2xxxx</t>
+  </si>
+  <si>
+    <t>Nguyen Van A</t>
+  </si>
+  <si>
+    <t>Personal matter</t>
+  </si>
+  <si>
+    <t>bo_phan</t>
+  </si>
+  <si>
+    <t>MIS</t>
   </si>
 </sst>
 </file>
@@ -101,13 +116,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -390,132 +411,214 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" customWidth="1"/>
+    <col min="3" max="4" width="15.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="5">
+        <v>46076</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E3" s="5"/>
+      <c r="F3" s="3"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E4" s="4"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E9" s="5"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E10" s="5"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E11" s="5"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E12" s="5"/>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E13" s="5"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E14" s="5"/>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E20" s="5"/>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E21" s="5"/>
+    </row>
+    <row r="22" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E22" s="5"/>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="5"/>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E24" s="5"/>
+    </row>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E25" s="5"/>
+    </row>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E26" s="5"/>
+    </row>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E27" s="5"/>
+    </row>
+    <row r="28" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E28" s="5"/>
+    </row>
+    <row r="29" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="5"/>
+    </row>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="5"/>
+    </row>
+    <row r="31" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E31" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>